<commit_message>
working updated benders cuts; remove mccormack from SP
</commit_message>
<xml_diff>
--- a/Model objective analysis/quantity discount/L_Shape_base_35_tender_fixed.xlsx
+++ b/Model objective analysis/quantity discount/L_Shape_base_35_tender_fixed.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,15 +452,15 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -473,15 +473,15 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
         <v>10</v>
@@ -494,18 +494,18 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -515,18 +515,18 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -536,15 +536,15 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
@@ -557,18 +557,18 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -578,18 +578,18 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -599,15 +599,15 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D9" t="n">
         <v>10</v>
@@ -620,20 +620,650 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mumps</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mumps</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>121</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HPV</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HPV</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>136</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HPV</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>153</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HPV</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>155</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HPV</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>172</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Hib</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>179</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Hib</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>199</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hib</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>212</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pertussis</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>219</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pertussis</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>239</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Pertussis</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>252</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>261</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>279</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>292</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>299</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>319</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>332</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>10</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>339</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>359</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>372</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>379</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>399</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>412</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>6</v>
+      </c>
+      <c r="D35" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>419</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>439</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>452</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>Rubella</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="C38" t="n">
+        <v>6</v>
+      </c>
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>459</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>478</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Full</t>
         </is>

</xml_diff>

<commit_message>
updated constraints, working SEC
</commit_message>
<xml_diff>
--- a/Model objective analysis/quantity discount/L_Shape_base_35_tender_fixed.xlsx
+++ b/Model objective analysis/quantity discount/L_Shape_base_35_tender_fixed.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -463,7 +463,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -473,7 +473,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -515,7 +515,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -523,10 +523,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -536,18 +536,18 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
         <v>6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>10</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -557,18 +557,18 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>PCV</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -599,18 +599,18 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -620,11 +620,11 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -641,18 +641,18 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>118</v>
+        <v>64</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -662,18 +662,18 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>121</v>
+        <v>66</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HPV</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -683,15 +683,15 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HPV</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
         <v>10</v>
@@ -704,18 +704,18 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>136</v>
+        <v>78</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HPV</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -725,18 +725,18 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>153</v>
+        <v>80</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HPV</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -746,18 +746,18 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>155</v>
+        <v>87</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HPV</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -767,18 +767,18 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>172</v>
+        <v>91</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hib</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>6</v>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -788,18 +788,18 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>179</v>
+        <v>97</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hib</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -809,18 +809,18 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>199</v>
+        <v>104</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hib</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -830,18 +830,18 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>212</v>
+        <v>106</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -851,18 +851,18 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>219</v>
+        <v>111</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -872,18 +872,18 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>239</v>
+        <v>118</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -893,18 +893,18 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>252</v>
+        <v>128</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rotavirus</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -914,18 +914,18 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>261</v>
+        <v>143</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rotavirus</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -935,18 +935,18 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>279</v>
+        <v>144</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rotavirus</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -956,18 +956,18 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>292</v>
+        <v>146</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Polio</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -977,18 +977,18 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>299</v>
+        <v>148</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Polio</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -998,18 +998,18 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>319</v>
+        <v>155</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Polio</t>
+          <t>HPV</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1019,18 +1019,18 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>332</v>
+        <v>166</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1040,18 +1040,18 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>339</v>
+        <v>172</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1061,18 +1061,18 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>359</v>
+        <v>178</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1082,18 +1082,18 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>372</v>
+        <v>182</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hepatitis_B</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1103,18 +1103,18 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>379</v>
+        <v>184</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hepatitis_B</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1124,18 +1124,18 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>399</v>
+        <v>188</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Hepatitis_B</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1145,18 +1145,18 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>412</v>
+        <v>190</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1166,18 +1166,18 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>419</v>
+        <v>199</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Hib</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1187,18 +1187,18 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>439</v>
+        <v>200</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1208,18 +1208,18 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>452</v>
+        <v>209</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1229,18 +1229,18 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>459</v>
+        <v>217</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1250,20 +1250,986 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>478</v>
+        <v>223</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
         <v>3</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>224</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Pertussis</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="n">
+        <v>10</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>239</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Pertussis</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>241</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>245</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>252</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>7</v>
+      </c>
+      <c r="D46" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>263</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>264</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>266</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>9</v>
+      </c>
+      <c r="D49" t="n">
+        <v>9</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>269</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" t="n">
+        <v>8</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>270</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>279</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Rotavirus</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>283</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+      <c r="D53" t="n">
+        <v>9</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>289</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4</v>
+      </c>
+      <c r="D54" t="n">
+        <v>8</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>295</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>7</v>
+      </c>
+      <c r="D55" t="n">
+        <v>7</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>305</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>9</v>
+      </c>
+      <c r="D57" t="n">
+        <v>10</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>312</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" t="n">
+        <v>6</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>319</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Polio</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>327</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>336</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>7</v>
+      </c>
+      <c r="D62" t="n">
+        <v>10</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>343</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>347</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>8</v>
+      </c>
+      <c r="D64" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>351</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>4</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>359</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Diphtheria</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>363</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>365</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>4</v>
+      </c>
+      <c r="D68" t="n">
+        <v>5</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>372</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>6</v>
+      </c>
+      <c r="D69" t="n">
+        <v>10</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>375</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>7</v>
+      </c>
+      <c r="D70" t="n">
+        <v>7</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>382</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>385</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>9</v>
+      </c>
+      <c r="D72" t="n">
+        <v>10</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>391</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>3</v>
+      </c>
+      <c r="D73" t="n">
+        <v>4</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>399</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Hepatitis_B</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>416</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>7</v>
+      </c>
+      <c r="D75" t="n">
+        <v>10</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>422</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>428</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>8</v>
+      </c>
+      <c r="D77" t="n">
+        <v>9</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>432</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>3</v>
+      </c>
+      <c r="D78" t="n">
+        <v>6</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>439</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>445</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>4</v>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>451</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="n">
+        <v>7</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>457</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>7</v>
+      </c>
+      <c r="D82" t="n">
+        <v>9</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>462</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>467</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>8</v>
+      </c>
+      <c r="D84" t="n">
+        <v>10</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>474</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>478</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>Full</t>
         </is>

</xml_diff>